<commit_message>
Fix: tambah spans attribute agar Excel dapat menampilkan data dengan benar
</commit_message>
<xml_diff>
--- a/Penerima Manfaat - Balita.xlsx
+++ b/Penerima Manfaat - Balita.xlsx
@@ -1625,7 +1625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1683,7 +1683,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>66</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>70</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>74</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>78</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>82</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>86</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>90</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>98</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>106</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>110</v>
       </c>
@@ -2005,7 +2005,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>114</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>118</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>122</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>126</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>130</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>137</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>141</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>145</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>149</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>153</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>156</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>160</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>164</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>168</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>172</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>176</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>180</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>184</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>192</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>196</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>200</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>204</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>208</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>212</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>216</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>220</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>226</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>230</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>234</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>238</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>242</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>246</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>46</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>251</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>51</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>256</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>260</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>264</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>268</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>272</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>276</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>280</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>284</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>288</v>
       </c>
@@ -3109,7 +3109,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>292</v>
       </c>
@@ -3132,7 +3132,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>296</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>300</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>304</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>308</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>312</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>316</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>320</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>324</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>328</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>332</v>
       </c>
@@ -3362,7 +3362,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>336</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>340</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>344</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>348</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>352</v>
       </c>
@@ -3477,7 +3477,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>356</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>359</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>363</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>367</v>
       </c>
@@ -3569,7 +3569,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>371</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>375</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>379</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>383</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>387</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>391</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>395</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>399</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>403</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>407</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>411</v>
       </c>
@@ -3822,7 +3822,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>415</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>419</v>
       </c>

</xml_diff>